<commit_message>
invoicing: match June invoice — fix dup pages, stray 0, signature rendering
- packager: export both invoice sheets in ONE job (LibreOffice was rendering both
  each time, duplicating pages 1-2). One summary+detail, merged once.
- template: blank detail A1 (was ='Invoice Summary'!B1 -> stray '0' top-left).
- signatures: revert to originals + transparent top margin (no trim/darken); scale
  invoice + timesheet signatures by INK height (aspect-preserved) so they render at
  the prior invoice's size and aren't clipped/squashed.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/invoicing/templates/HDR_template.xlsx
+++ b/invoicing/templates/HDR_template.xlsx
@@ -2811,10 +2811,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:18" s="16" customFormat="1" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A1" s="60">
-        <f>'Invoice Summary'!B1</f>
-        <v>0</v>
-      </c>
+      <c r="A1"/>
       <c r="L1" s="17"/>
       <c r="M1" s="17"/>
       <c r="N1" s="17"/>

</xml_diff>